<commit_message>
Added new RDF data schemes and visual schemes for employment-table06-08, fixed XLSX spreadsheet for employment-table06
</commit_message>
<xml_diff>
--- a/sources/table_normalization/xlsx/employment-table06.xlsx
+++ b/sources/table_normalization/xlsx/employment-table06.xlsx
@@ -149,11 +149,11 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -473,46 +473,46 @@
       <c r="I1" s="3"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A5" s="2"/>
-      <c r="B5" s="1" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1" t="s">
+      <c r="C5" s="4"/>
+      <c r="D5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1" t="s">
+      <c r="E5" s="4"/>
+      <c r="F5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1" t="s">
+      <c r="G5" s="4"/>
+      <c r="H5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="I5" s="1"/>
+      <c r="I5" s="4"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" s="2"/>
+      <c r="A6" s="5"/>
       <c r="B6">
         <v>2022</v>
       </c>
@@ -544,7 +544,7 @@
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" s="5" t="s">
+      <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B9">
@@ -573,7 +573,7 @@
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A10" s="5" t="s">
+      <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B10">
@@ -602,7 +602,7 @@
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B11">
@@ -631,7 +631,7 @@
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A12" s="5" t="s">
+      <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B12">
@@ -660,7 +660,7 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A13" s="5" t="s">
+      <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B13">
@@ -689,7 +689,7 @@
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B14">
@@ -718,7 +718,7 @@
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A15" s="5" t="s">
+      <c r="A15" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B15">
@@ -747,7 +747,7 @@
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A16" s="5" t="s">
+      <c r="A16" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B16">
@@ -781,7 +781,7 @@
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A19" s="5" t="s">
+      <c r="A19" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B19">
@@ -810,7 +810,7 @@
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A20" s="5" t="s">
+      <c r="A20" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B20">
@@ -839,7 +839,7 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A21" s="5" t="s">
+      <c r="A21" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B21">
@@ -868,7 +868,7 @@
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A22" s="5" t="s">
+      <c r="A22" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B22">
@@ -897,7 +897,7 @@
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A23" s="5" t="s">
+      <c r="A23" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B23">
@@ -926,7 +926,7 @@
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A24" s="5" t="s">
+      <c r="A24" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B24">
@@ -955,7 +955,7 @@
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A25" s="5" t="s">
+      <c r="A25" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B25">
@@ -984,7 +984,7 @@
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A26" s="5" t="s">
+      <c r="A26" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B26">
@@ -1018,7 +1018,7 @@
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A29" s="5" t="s">
+      <c r="A29" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B29">
@@ -1047,7 +1047,7 @@
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A30" s="5" t="s">
+      <c r="A30" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B30">
@@ -1076,7 +1076,7 @@
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A31" s="5" t="s">
+      <c r="A31" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B31">
@@ -1105,7 +1105,7 @@
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A32" s="5" t="s">
+      <c r="A32" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B32">
@@ -1134,7 +1134,7 @@
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A33" s="5" t="s">
+      <c r="A33" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B33">
@@ -1163,7 +1163,7 @@
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A34" s="5" t="s">
+      <c r="A34" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B34">
@@ -1192,7 +1192,7 @@
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A35" s="5" t="s">
+      <c r="A35" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B35">
@@ -1221,7 +1221,7 @@
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A36" s="5" t="s">
+      <c r="A36" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B36">
@@ -1255,7 +1255,7 @@
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A39" s="5" t="s">
+      <c r="A39" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B39">
@@ -1284,7 +1284,7 @@
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A40" s="5" t="s">
+      <c r="A40" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B40">
@@ -1313,7 +1313,7 @@
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A41" s="5" t="s">
+      <c r="A41" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B41">
@@ -1342,7 +1342,7 @@
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B42">
@@ -1371,7 +1371,7 @@
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A43" s="5" t="s">
+      <c r="A43" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B43">
@@ -1400,7 +1400,7 @@
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A44" s="5" t="s">
+      <c r="A44" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B44">
@@ -1429,7 +1429,7 @@
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A45" s="5" t="s">
+      <c r="A45" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B45">
@@ -1458,7 +1458,7 @@
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A46" s="5" t="s">
+      <c r="A46" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B46">
@@ -1492,7 +1492,7 @@
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A49" s="5" t="s">
+      <c r="A49" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B49">
@@ -1521,7 +1521,7 @@
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A50" s="5" t="s">
+      <c r="A50" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B50">
@@ -1550,7 +1550,7 @@
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A51" s="5" t="s">
+      <c r="A51" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B51">
@@ -1579,7 +1579,7 @@
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A52" s="5" t="s">
+      <c r="A52" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B52">
@@ -1608,7 +1608,7 @@
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A53" s="5" t="s">
+      <c r="A53" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B53">
@@ -1637,7 +1637,7 @@
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A54" s="5" t="s">
+      <c r="A54" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B54">
@@ -1666,7 +1666,7 @@
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A55" s="5" t="s">
+      <c r="A55" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B55">
@@ -1695,7 +1695,7 @@
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A56" s="5" t="s">
+      <c r="A56" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B56">
@@ -1729,7 +1729,7 @@
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A59" s="5" t="s">
+      <c r="A59" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B59">
@@ -1758,7 +1758,7 @@
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A60" s="5" t="s">
+      <c r="A60" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B60">
@@ -1787,7 +1787,7 @@
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A61" s="5" t="s">
+      <c r="A61" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B61">
@@ -1816,7 +1816,7 @@
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A62" s="5" t="s">
+      <c r="A62" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B62">
@@ -1845,7 +1845,7 @@
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A63" s="5" t="s">
+      <c r="A63" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B63">
@@ -1874,7 +1874,7 @@
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A64" s="5" t="s">
+      <c r="A64" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B64">
@@ -1903,7 +1903,7 @@
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A65" s="5" t="s">
+      <c r="A65" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B65">
@@ -1932,7 +1932,7 @@
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A66" s="5" t="s">
+      <c r="A66" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B66">

</xml_diff>